<commit_message>
revision de CA de HU 1 y 2, creacion de usuarios de distintos roles para pruebas
</commit_message>
<xml_diff>
--- a/data/excel/activos.xlsx
+++ b/data/excel/activos.xlsx
@@ -110,6 +110,81 @@
   </x:si>
   <x:si>
     <x:t>2026-07-02T01:51:10.0285539Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CFA-1000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AUGER-1000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Camión Fábrica</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASTRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HD9 84.48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TWCK-41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>91</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-08T15:59:47.8384370Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-08T16:06:32.3858031Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRUEBA-2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>prueba-2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FAE_AND</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Unavailable</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SERV-04-18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No disponible</x:t>
+  </x:si>
+  <x:si>
+    <x:t>73</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-08T16:01:46.0338399Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-08T16:03:02.8111754Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRUEBA-3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>prueba-3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FAE_ESV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SERV-04-19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>64</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-08T16:15:43.3865096Z</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -475,17 +550,19 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:T2"/>
+  <x:dimension ref="A1:T5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="8.282054" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.710625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="12.710625" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.282054" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11.139196" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="22.710625" style="0" customWidth="1"/>
-    <x:col min="7" max="8" width="7.424911" style="0" customWidth="1"/>
-    <x:col min="9" max="10" width="7.996339" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.424911" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="9.853482" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8.996339" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="12.710625" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="10.139196" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="9.282054" style="0" customWidth="1"/>
@@ -618,6 +695,153 @@
         <x:v>31</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" spans="1:20">
+      <x:c r="A3" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="L3" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M3" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="N3" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="O3" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="P3" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="Q3" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="S3" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="T3" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:20">
+      <x:c r="A4" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L4" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M4" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="N4" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="O4" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="P4" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="Q4" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="S4" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="T4" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:20">
+      <x:c r="A5" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="L5" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M5" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="N5" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="O5" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="P5" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="Q5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="S5" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="T5" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>